<commit_message>
Add "Drone" short and a new jerky icon to the board
New row: DRONE (15 min, tastes like "a drone with free will"),
linking to https://www.youtube.com/watch?v=RubSLGTrdOA. Paired with
an original hand-drawn beef jerky SVG (transparent bg) since none of
the existing food art fit an unused slot.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MRRrbWVCmuuHE8Hg1SqHXz
</commit_message>
<xml_diff>
--- a/shorts.xlsx
+++ b/shorts.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="shorts" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="shorts" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -332,7 +332,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="36" customWidth="1" style="5" min="1" max="1"/>
@@ -547,7 +547,7 @@
           <t>being in the wrong place at the wrong time</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="0" t="inlineStr">
         <is>
           <t>Cheese_1.svg</t>
         </is>
@@ -574,7 +574,7 @@
           <t>getting dumped by your AI girlfriend</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="0" t="inlineStr">
         <is>
           <t>Cheese_2.svg</t>
         </is>
@@ -601,7 +601,7 @@
           <t>a pretty road trip monologue</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="0" t="inlineStr">
         <is>
           <t>Crackers.svg</t>
         </is>
@@ -628,7 +628,7 @@
           <t>a Chat GPT conversation gone wrong</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="0" t="inlineStr">
         <is>
           <t>Honey.svg</t>
         </is>
@@ -655,7 +655,7 @@
           <t>rainy warehouse bullets</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="0" t="inlineStr">
         <is>
           <t>Olives.svg</t>
         </is>
@@ -682,7 +682,7 @@
           <t>the Matrix in a red motorcyle helmet</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="0" t="inlineStr">
         <is>
           <t>Purple_Grapes.svg</t>
         </is>
@@ -709,7 +709,7 @@
           <t>a space desert jedi training session</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="0" t="inlineStr">
         <is>
           <t>Sausage_3.svg</t>
         </is>
@@ -717,6 +717,33 @@
       <c r="E14" s="3" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=H08tGjXNHO4</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Drone</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>15 min</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>a drone with free will</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Beef_Jerky.svg</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=RubSLGTrdOA</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add "The Moon Before Us" short and a fig icon to the board
New row: THE MOON BEFORE US (4 min, tastes like "the History
Channel"), linking to https://www.youtube.com/watch?v=3RXi5QFhjuU.
Paired with an original fig cross-section SVG (transparent bg).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MRRrbWVCmuuHE8Hg1SqHXz
</commit_message>
<xml_diff>
--- a/shorts.xlsx
+++ b/shorts.xlsx
@@ -332,7 +332,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="36" customWidth="1" style="5" min="1" max="1"/>
@@ -721,29 +721,56 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="0" t="inlineStr">
         <is>
           <t>Drone</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="0" t="inlineStr">
         <is>
           <t>15 min</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="0" t="inlineStr">
         <is>
           <t>a drone with free will</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="0" t="inlineStr">
         <is>
           <t>Beef_Jerky.svg</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E15" s="0" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=RubSLGTrdOA</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>The Moon Before Us</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>4 min</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>the History Channel</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Fig.svg</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=3RXi5QFhjuU</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add "The God Man" short and a walnut icon to the board
New row: THE GOD MAN (10 min, tastes like "a researcher's log"),
linking to https://www.youtube.com/watch?v=WY9CTDM3l4M. Paired with
an original cracked walnut SVG (transparent bg).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MRRrbWVCmuuHE8Hg1SqHXz
</commit_message>
<xml_diff>
--- a/shorts.xlsx
+++ b/shorts.xlsx
@@ -332,7 +332,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="36" customWidth="1" style="5" min="1" max="1"/>
@@ -748,29 +748,56 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="0" t="inlineStr">
         <is>
           <t>The Moon Before Us</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="0" t="inlineStr">
         <is>
           <t>4 min</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="0" t="inlineStr">
         <is>
           <t>the History Channel</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="0" t="inlineStr">
         <is>
           <t>Fig.svg</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E16" s="0" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=3RXi5QFhjuU</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>The God Man</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>10 min</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>a researcher's log</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Walnut.svg</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=WY9CTDM3l4M</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add September viewed section with locked stars; drop eaten state
Rows in shorts.xlsx with a `viewed` month now render below a "we viewed
these in <month>" divider, with read-only stars from the new `stars`
column. Adds "There Is No Antimemetics Division". Removes the
eaten/unclickable behavior so every card can be clicked repeatedly.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014ejeBEpPZXZLW9oRgPcZZZ
</commit_message>
<xml_diff>
--- a/shorts.xlsx
+++ b/shorts.xlsx
@@ -332,7 +332,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="36" customWidth="1" style="5" min="1" max="1"/>
@@ -368,6 +368,16 @@
           <t>url</t>
         </is>
       </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>viewed</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>stars</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -395,6 +405,14 @@
           <t>https://www.youtube.com/watch?v=NLAZubEa6X4</t>
         </is>
       </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>September</t>
+        </is>
+      </c>
+      <c r="G2" s="2">
+        <v>4</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -449,6 +467,14 @@
           <t>https://www.youtube.com/watch?v=Wln5dlYKA1k</t>
         </is>
       </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>September</t>
+        </is>
+      </c>
+      <c r="G4" s="2">
+        <v>4</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -476,6 +502,14 @@
           <t>https://www.youtube.com/watch?v=cLpvMRMnjQc</t>
         </is>
       </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>September</t>
+        </is>
+      </c>
+      <c r="G5" s="2">
+        <v>3</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -503,6 +537,14 @@
           <t>https://www.youtube.com/watch?v=wncYbIpm6hk</t>
         </is>
       </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>September</t>
+        </is>
+      </c>
+      <c r="G6" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -557,6 +599,14 @@
           <t>https://www.youtube.com/watch?v=dYAHOZ_91A0&amp;time_continue=599&amp;source_ve_path=NzY3NTg&amp;embeds_referring_euri=https%3A%2F%2Fwww.filmcrux.com%2F</t>
         </is>
       </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>September</t>
+        </is>
+      </c>
+      <c r="G8" s="2">
+        <v>3</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -692,6 +742,14 @@
           <t>https://www.youtube.com/watch?v=IOqUOrtPXlQ</t>
         </is>
       </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>September</t>
+        </is>
+      </c>
+      <c r="G13" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -719,6 +777,14 @@
           <t>https://www.youtube.com/watch?v=H08tGjXNHO4</t>
         </is>
       </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>September</t>
+        </is>
+      </c>
+      <c r="G14" s="2">
+        <v>2</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
@@ -746,6 +812,14 @@
           <t>https://www.youtube.com/watch?v=RubSLGTrdOA</t>
         </is>
       </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>September</t>
+        </is>
+      </c>
+      <c r="G15" s="2">
+        <v>3</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
@@ -772,6 +846,14 @@
         <is>
           <t>https://www.youtube.com/watch?v=3RXi5QFhjuU</t>
         </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>September</t>
+        </is>
+      </c>
+      <c r="G16" s="2">
+        <v>5</v>
       </c>
     </row>
     <row r="17">
@@ -1781,6 +1863,41 @@
     <row r="998" ht="15.75" customHeight="1" s="5"/>
     <row r="999" ht="15.75" customHeight="1" s="5"/>
     <row r="1000" ht="15.75" customHeight="1" s="5"/>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>There Is No Antimemetics Division</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>food_olive.svg</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>September</t>
+        </is>
+      </c>
+      <c r="G18" s="2">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>

</xml_diff>

<commit_message>
Add "Dynamo Dream" and "Crash Site" shorts to the board
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014ejeBEpPZXZLW9oRgPcZZZ
</commit_message>
<xml_diff>
--- a/shorts.xlsx
+++ b/shorts.xlsx
@@ -332,7 +332,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="36" customWidth="1" style="5" min="1" max="1"/>
@@ -1898,6 +1898,60 @@
         <v>3</v>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Dynamo Dream</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>22 min</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Blade Runner built in Blender</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Honey.svg</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=LsGZ_2RuJ2A</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Crash Site</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>14 min</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>a hiking trip that turns into first contact</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Walnut.svg</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=HFxEYlyt0po</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>

</xml_diff>

<commit_message>
Link "There Is No Antimemetics Division" to its YouTube video
Adds the DUST film's url, length and a tastes-like note.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014ejeBEpPZXZLW9oRgPcZZZ
</commit_message>
<xml_diff>
--- a/shorts.xlsx
+++ b/shorts.xlsx
@@ -1871,12 +1871,12 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>16 min</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>a memory you can't hold onto</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -1884,9 +1884,9 @@
           <t>food_olive.svg</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t/>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=3v8AsTHfAG0</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Add "They Weren't Supposed To Appear" short and reuse the Fig icon
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NCTEDuTTKv2Xk9hdCH1vNG
</commit_message>
<xml_diff>
--- a/shorts.xlsx
+++ b/shorts.xlsx
@@ -332,7 +332,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="36" customWidth="1" style="5" min="1" max="1"/>
@@ -410,7 +410,7 @@
           <t>September</t>
         </is>
       </c>
-      <c r="G2" s="2">
+      <c r="G2" s="2" t="n">
         <v>4</v>
       </c>
     </row>
@@ -472,7 +472,7 @@
           <t>September</t>
         </is>
       </c>
-      <c r="G4" s="2">
+      <c r="G4" s="2" t="n">
         <v>4</v>
       </c>
     </row>
@@ -507,7 +507,7 @@
           <t>September</t>
         </is>
       </c>
-      <c r="G5" s="2">
+      <c r="G5" s="2" t="n">
         <v>3</v>
       </c>
     </row>
@@ -542,7 +542,7 @@
           <t>September</t>
         </is>
       </c>
-      <c r="G6" s="2">
+      <c r="G6" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -604,7 +604,7 @@
           <t>September</t>
         </is>
       </c>
-      <c r="G8" s="2">
+      <c r="G8" s="2" t="n">
         <v>3</v>
       </c>
     </row>
@@ -747,7 +747,7 @@
           <t>September</t>
         </is>
       </c>
-      <c r="G13" s="2">
+      <c r="G13" s="2" t="n">
         <v>2</v>
       </c>
     </row>
@@ -782,7 +782,7 @@
           <t>September</t>
         </is>
       </c>
-      <c r="G14" s="2">
+      <c r="G14" s="2" t="n">
         <v>2</v>
       </c>
     </row>
@@ -817,7 +817,7 @@
           <t>September</t>
         </is>
       </c>
-      <c r="G15" s="2">
+      <c r="G15" s="2" t="n">
         <v>3</v>
       </c>
     </row>
@@ -852,38 +852,153 @@
           <t>September</t>
         </is>
       </c>
-      <c r="G16" s="2">
+      <c r="G16" s="2" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="0" t="inlineStr">
         <is>
           <t>The God Man</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="0" t="inlineStr">
         <is>
           <t>10 min</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="0" t="inlineStr">
         <is>
           <t>a researcher's log</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="0" t="inlineStr">
         <is>
           <t>Walnut.svg</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E17" s="0" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=WY9CTDM3l4M</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="15.75" customHeight="1" s="5"/>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>There Is No Antimemetics Division</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>16 min</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>a memory you can't hold onto</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>food_olive.svg</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=3v8AsTHfAG0</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>September</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Dynamo Dream</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>22 min</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Blade Runner built in Blender</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Honey.svg</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=LsGZ_2RuJ2A</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Crash Site</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>14 min</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>a hiking trip that turns into first contact</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Walnut.svg</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=HFxEYlyt0po</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15.75" customHeight="1" s="5">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>They Weren't Supposed To Appear</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>5 min</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>the History Channel 2</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Fig.svg</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=9DymCrfcRdY</t>
+        </is>
+      </c>
+    </row>
     <row r="22" ht="15.75" customHeight="1" s="5"/>
     <row r="23" ht="15.75" customHeight="1" s="5"/>
     <row r="24" ht="15.75" customHeight="1" s="5"/>
@@ -1863,95 +1978,6 @@
     <row r="998" ht="15.75" customHeight="1" s="5"/>
     <row r="999" ht="15.75" customHeight="1" s="5"/>
     <row r="1000" ht="15.75" customHeight="1" s="5"/>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>There Is No Antimemetics Division</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>16 min</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>a memory you can't hold onto</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>food_olive.svg</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=3v8AsTHfAG0</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>September</t>
-        </is>
-      </c>
-      <c r="G18" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Dynamo Dream</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>22 min</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Blade Runner built in Blender</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>Honey.svg</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=LsGZ_2RuJ2A</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Crash Site</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>14 min</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>a hiking trip that turns into first contact</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>Walnut.svg</t>
-        </is>
-      </c>
-      <c r="E20" s="3" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=HFxEYlyt0po</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>

</xml_diff>